<commit_message>
chore: project update 2026-07-29 (2) -- fresh NBG spot balance EUR58,805, reconciliation residual normalized to EUR787.94
</commit_message>
<xml_diff>
--- a/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
+++ b/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
@@ -32,7 +32,7 @@
     <t xml:space="preserve">Ag. Nikolaos Home — Project Balance Sheet</t>
   </si>
   <si>
-    <t xml:space="preserve">Financial ground truth. Currency: EUR. Last updated 2026-07-21. Sources: project folder, Drive payments sheet, WhatsApp 'Evia HOME', Gmail, bank confirmations.</t>
+    <t xml:space="preserve">Financial ground truth. Currency: EUR. Last updated 2026-07-29. Sources: project folder, Drive payments sheet, WhatsApp 'Evia HOME', Gmail, bank confirmations.</t>
   </si>
   <si>
     <t xml:space="preserve">FUNDING &amp; POSITION</t>
@@ -53,7 +53,7 @@
     <t xml:space="preserve">Current NBG balance</t>
   </si>
   <si>
-    <t xml:space="preserve">Reported 2026-07-21 (see Reconciliation &gt; Rolling Bridge for the residual check)</t>
+    <t xml:space="preserve">Reported 2026-07-29 (see Reconciliation &gt; Rolling Bridge for the residual check)</t>
   </si>
   <si>
     <t xml:space="preserve">RENOVATION</t>
@@ -1331,7 +1331,7 @@
     <t xml:space="preserve">Computed balance (bridge)</t>
   </si>
   <si>
-    <t xml:space="preserve">Reported balance (2026-07-21)</t>
+    <t xml:space="preserve">Reported balance (2026-07-29)</t>
   </si>
   <si>
     <t xml:space="preserve">Residual (bridge − reported)</t>
@@ -2225,7 +2225,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="8" t="n">
-        <v>65505</v>
+        <v>58805</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>8</v>
@@ -8051,7 +8051,7 @@
         <v>434</v>
       </c>
       <c r="C31" s="48" t="n">
-        <v>65505</v>
+        <v>58805</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8060,7 +8060,7 @@
       </c>
       <c r="C32" s="49" t="n">
         <f aca="false">C30-C31</f>
-        <v>-5912.06</v>
+        <v>787.940000000002</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
chore: project update 2026-09-15 -- work resumes after extended pause, EUR400 water fee (payment declined) logged as Committed
</commit_message>
<xml_diff>
--- a/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
+++ b/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId3"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1501" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1508" uniqueCount="487">
   <si>
     <t xml:space="preserve">Ag. Nikolaos Home — Project Balance Sheet</t>
   </si>
@@ -867,6 +867,18 @@
   </si>
   <si>
     <t xml:space="preserve">Kairis - partial payment toward column/beam debt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Water connection fee (mains) + water meter purchase - one-off, now connected to mains supply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accountant (POS transfer attempted Sep 12, declined - payment method to be resolved)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pending</t>
   </si>
   <si>
     <t xml:space="preserve">PAID — total</t>
@@ -2244,7 +2256,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="9" t="n">
-        <f aca="false">'Renovation Ledger'!E153</f>
+        <f aca="false">'Renovation Ledger'!E154</f>
         <v>99161.47</v>
       </c>
       <c r="C10" s="6" t="s">
@@ -2256,8 +2268,8 @@
         <v>12</v>
       </c>
       <c r="B11" s="10" t="n">
-        <f aca="false">'Renovation Ledger'!E154</f>
-        <v>20178</v>
+        <f aca="false">'Renovation Ledger'!E155</f>
+        <v>20578</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>13</v>
@@ -2268,7 +2280,7 @@
         <v>14</v>
       </c>
       <c r="B12" s="5" t="n">
-        <f aca="false">'Property Acquisition 2025'!D19+'Renovation Ledger'!E153</f>
+        <f aca="false">'Property Acquisition 2025'!D19+'Renovation Ledger'!E154</f>
         <v>270870.47</v>
       </c>
       <c r="C12" s="6" t="s">
@@ -2327,7 +2339,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I156"/>
+  <dimension ref="A1:I157"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="13"/>
@@ -6667,39 +6679,66 @@
         <v>272</v>
       </c>
     </row>
-    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D153" s="19" t="s">
+    <row r="153" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="14" t="s">
         <v>280</v>
       </c>
-      <c r="E153" s="20" t="n">
-        <f aca="false">SUMIF(H5:H152,"Paid",E5:E152)</f>
-        <v>99161.47</v>
-      </c>
+      <c r="B153" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="C153" s="14" t="s">
+        <v>281</v>
+      </c>
+      <c r="D153" s="14" t="s">
+        <v>282</v>
+      </c>
+      <c r="E153" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="F153" s="16" t="s">
+        <v>283</v>
+      </c>
+      <c r="G153" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="H153" s="18" t="s">
+        <v>264</v>
+      </c>
+      <c r="I153" s="14"/>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D154" s="19" t="s">
-        <v>281</v>
-      </c>
-      <c r="E154" s="21" t="n">
-        <f aca="false">SUMIF(H5:H152,"Committed",E5:E152)</f>
-        <v>20178</v>
+        <v>284</v>
+      </c>
+      <c r="E154" s="20" t="n">
+        <f aca="false">SUMIF(H5:H153,"Paid",E5:E153)</f>
+        <v>99161.47</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D155" s="22" t="s">
-        <v>282</v>
-      </c>
-      <c r="E155" s="23" t="n">
-        <f aca="false">SUMIFS(E5:E152,H5:H152,"Paid",G5:G152,"Yes")</f>
-        <v>97133.92</v>
+      <c r="D155" s="19" t="s">
+        <v>285</v>
+      </c>
+      <c r="E155" s="21" t="n">
+        <f aca="false">SUMIF(H5:H153,"Committed",E5:E153)</f>
+        <v>20578</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D156" s="22" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E156" s="23" t="n">
-        <f aca="false">SUMIFS(E5:E152,H5:H152,"Paid",G5:G152,"No")</f>
+        <f aca="false">SUMIFS(E5:E153,H5:H153,"Paid",G5:G153,"Yes")</f>
+        <v>97133.92</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D157" s="22" t="s">
+        <v>287</v>
+      </c>
+      <c r="E157" s="23" t="n">
+        <f aca="false">SUMIFS(E5:E153,H5:H153,"Paid",G5:G153,"No")</f>
         <v>2027.55</v>
       </c>
     </row>
@@ -6735,7 +6774,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6744,7 +6783,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6753,33 +6792,33 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="B5" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="E5" s="17" t="s">
         <v>36</v>
@@ -6787,16 +6826,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="B6" s="24" t="n">
         <v>15000</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="E6" s="17" t="s">
         <v>36</v>
@@ -6804,16 +6843,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="B7" s="24" t="n">
         <v>130000</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="E7" s="17" t="s">
         <v>36</v>
@@ -6821,16 +6860,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="B8" s="24" t="n">
         <v>10000</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="E8" s="17" t="s">
         <v>36</v>
@@ -6838,16 +6877,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B9" s="24" t="n">
         <v>20000</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="E9" s="17" t="s">
         <v>36</v>
@@ -6855,16 +6894,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="B10" s="24" t="n">
         <v>70000</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>36</v>
@@ -6872,16 +6911,16 @@
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="B11" s="24" t="n">
         <v>2000</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="E11" s="18" t="s">
         <v>183</v>
@@ -6889,16 +6928,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="B12" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="E12" s="17" t="s">
         <v>36</v>
@@ -6906,7 +6945,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="25" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="B13" s="26" t="n">
         <f aca="false">SUMIF(E5:E12,"Yes",B5:B12)</f>
@@ -6915,7 +6954,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="27" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="B15" s="27"/>
       <c r="C15" s="27"/>
@@ -6924,7 +6963,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="27" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="B16" s="27"/>
       <c r="C16" s="27"/>
@@ -6966,7 +7005,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6975,7 +7014,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6984,13 +7023,13 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>26</v>
@@ -6999,18 +7038,18 @@
         <v>28</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="D5" s="24" t="n">
         <v>18500</v>
@@ -7019,18 +7058,18 @@
         <v>36</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="D6" s="24" t="n">
         <v>107000</v>
@@ -7039,18 +7078,18 @@
         <v>36</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="D7" s="24" t="n">
         <v>19731</v>
@@ -7059,18 +7098,18 @@
         <v>36</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="D8" s="24" t="n">
         <v>7410</v>
@@ -7079,18 +7118,18 @@
         <v>36</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D9" s="24" t="n">
         <v>4350</v>
@@ -7099,15 +7138,15 @@
         <v>36</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>150</v>
@@ -7119,15 +7158,15 @@
         <v>36</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="C11" s="14" t="s">
         <v>150</v>
@@ -7139,18 +7178,18 @@
         <v>36</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="D12" s="24" t="n">
         <v>2490</v>
@@ -7159,18 +7198,18 @@
         <v>36</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="D13" s="24" t="n">
         <v>800</v>
@@ -7179,18 +7218,18 @@
         <v>36</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="D14" s="24" t="n">
         <v>520</v>
@@ -7202,13 +7241,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="D15" s="24" t="n">
         <v>680</v>
@@ -7220,13 +7259,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="D16" s="24" t="n">
         <v>3000</v>
@@ -7235,15 +7274,15 @@
         <v>36</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>48</v>
@@ -7255,15 +7294,15 @@
         <v>183</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C18" s="14" t="s">
         <v>48</v>
@@ -7275,12 +7314,12 @@
         <v>183</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C19" s="25" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="D19" s="26" t="n">
         <f aca="false">SUM(D5:D18)</f>
@@ -7289,7 +7328,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C20" s="19" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="D20" s="28" t="n">
         <f aca="false">SUMIF(E5:E18,"Yes",D5:D18)</f>
@@ -7298,7 +7337,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="27" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="27"/>
@@ -7339,7 +7378,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7348,7 +7387,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7357,10 +7396,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>27</v>
@@ -7369,7 +7408,7 @@
         <v>26</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7377,7 +7416,7 @@
         <v>170</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>182</v>
@@ -7386,7 +7425,7 @@
         <v>614</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7394,7 +7433,7 @@
         <v>205</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>208</v>
@@ -7403,7 +7442,7 @@
         <v>972.55</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7411,7 +7450,7 @@
         <v>212</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>182</v>
@@ -7420,7 +7459,7 @@
         <v>286</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7428,7 +7467,7 @@
         <v>216</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="C8" s="14" t="s">
         <v>208</v>
@@ -7437,12 +7476,12 @@
         <v>155</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="19" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="D9" s="20" t="n">
         <f aca="false">SUM(D5:D8)</f>
@@ -7451,7 +7490,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
@@ -7460,10 +7499,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>27</v>
@@ -7472,7 +7511,7 @@
         <v>26</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7480,16 +7519,16 @@
         <v>216</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="D13" s="15" t="n">
         <v>972.55</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
     </row>
   </sheetData>
@@ -7523,7 +7562,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7531,7 +7570,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7542,13 +7581,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7556,14 +7595,14 @@
         <v>38</v>
       </c>
       <c r="B5" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A5,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A5,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>30190</v>
       </c>
       <c r="C5" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7571,14 +7610,14 @@
         <v>51</v>
       </c>
       <c r="B6" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A6,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A6,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>37057.87</v>
       </c>
       <c r="C6" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7586,14 +7625,14 @@
         <v>106</v>
       </c>
       <c r="B7" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A7,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A7,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>7119</v>
       </c>
       <c r="C7" s="24" t="n">
         <v>9000</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7601,14 +7640,14 @@
         <v>43</v>
       </c>
       <c r="B8" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A8,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A8,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>2325</v>
       </c>
       <c r="C8" s="24" t="n">
         <v>11250</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7616,14 +7655,14 @@
         <v>82</v>
       </c>
       <c r="B9" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A9,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A9,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>4300</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>6000</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7631,14 +7670,14 @@
         <v>104</v>
       </c>
       <c r="B10" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A10,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A10,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>4225</v>
       </c>
       <c r="C10" s="24" t="n">
         <v>4500</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7646,14 +7685,14 @@
         <v>123</v>
       </c>
       <c r="B11" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A11,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A11,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>1550</v>
       </c>
       <c r="C11" s="24" t="n">
         <v>18700</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7661,14 +7700,14 @@
         <v>32</v>
       </c>
       <c r="B12" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A12,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A12,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>2097</v>
       </c>
       <c r="C12" s="24" t="n">
         <v>2000</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7676,14 +7715,14 @@
         <v>213</v>
       </c>
       <c r="B13" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A13,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A13,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>286</v>
       </c>
       <c r="C13" s="24" t="n">
         <v>25500</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7691,14 +7730,14 @@
         <v>219</v>
       </c>
       <c r="B14" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A14,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A14,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>905</v>
       </c>
       <c r="C14" s="24" t="n">
         <v>1000</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7706,14 +7745,14 @@
         <v>77</v>
       </c>
       <c r="B15" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A15,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A15,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>7666</v>
       </c>
       <c r="C15" s="24" t="n">
         <v>11350</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7721,14 +7760,14 @@
         <v>95</v>
       </c>
       <c r="B16" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A16,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A16,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>300</v>
       </c>
       <c r="C16" s="24" t="n">
         <v>5000</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7736,7 +7775,7 @@
         <v>71</v>
       </c>
       <c r="B17" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A17,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A17,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>270</v>
       </c>
       <c r="C17" s="24" t="n">
@@ -7751,14 +7790,14 @@
         <v>46</v>
       </c>
       <c r="B18" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A18,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A18,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>770.6</v>
       </c>
       <c r="C18" s="24" t="n">
         <v>500</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7766,19 +7805,19 @@
         <v>66</v>
       </c>
       <c r="B19" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E152,'Renovation Ledger'!B5:B152,A19,'Renovation Ledger'!H5:H152,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A19,'Renovation Ledger'!H5:H153,"Paid")</f>
         <v>100</v>
       </c>
       <c r="C19" s="24" t="n">
         <v>300</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="29" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="B20" s="20" t="n">
         <f aca="false">SUM(B5:B19)</f>
@@ -7820,7 +7859,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7828,7 +7867,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7836,106 +7875,106 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="30" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="C5" s="31" t="n">
         <v>21066.81</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="33" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="C6" s="34" t="n">
         <v>230000</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="35" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="C7" s="36" t="n">
         <v>-139459.28</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="35" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="C8" s="36" t="n">
         <v>-6350</v>
       </c>
       <c r="D8" s="32" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="35" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="C9" s="36" t="n">
         <v>-64730</v>
       </c>
       <c r="D9" s="32" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="35" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C10" s="36" t="n">
         <v>-4494.92</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="35" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="C11" s="36" t="n">
         <v>-711</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="35" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="C12" s="36" t="n">
         <v>-104.17</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="35" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="C13" s="36" t="n">
         <v>-14.5</v>
       </c>
       <c r="D13" s="32" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="29" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="C14" s="37" t="n">
         <f aca="false">SUM(C5:C13)</f>
@@ -7944,7 +7983,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="29" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="C15" s="38" t="n">
         <v>35202.94</v>
@@ -7952,7 +7991,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="39" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="C16" s="40" t="n">
         <f aca="false">C14-C15</f>
@@ -7961,21 +8000,21 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="29" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="41" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="C19" s="42" t="n">
-        <f aca="false">'Renovation Ledger'!E155</f>
+        <f aca="false">'Renovation Ledger'!E156</f>
         <v>97133.92</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="41" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="C20" s="42" t="n">
         <v>69935.92</v>
@@ -7983,37 +8022,37 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="43" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="C21" s="44" t="n">
-        <f aca="false">'Renovation Ledger'!E155-69935.92</f>
+        <f aca="false">'Renovation Ledger'!E156-69935.92</f>
         <v>27198</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="45" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="C23" s="45"/>
       <c r="D23" s="45"/>
     </row>
     <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="45" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="C24" s="45"/>
       <c r="D24" s="45"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="46" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="C26" s="46"/>
       <c r="D26" s="46"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="41" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="C27" s="42" t="n">
         <v>35202.94</v>
@@ -8021,7 +8060,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="41" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="C28" s="42" t="n">
         <f aca="false">SUMPRODUCT(('Funding (NBG Deposits)'!A5:A12&gt;"2026-06-25")*('Funding (NBG Deposits)'!E5:E12="Yes")*'Funding (NBG Deposits)'!B5:B12)</f>
@@ -8030,16 +8069,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="41" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="C29" s="42" t="n">
-        <f aca="false">SUMPRODUCT(('Renovation Ledger'!I5:I152&gt;"2026-06-25")*('Renovation Ledger'!H5:H152="Paid")*('Renovation Ledger'!G5:G152="Yes")*'Renovation Ledger'!E5:E152)</f>
+        <f aca="false">SUMPRODUCT(('Renovation Ledger'!I5:I153&gt;"2026-06-25")*('Renovation Ledger'!H5:H153="Paid")*('Renovation Ledger'!G5:G153="Yes")*'Renovation Ledger'!E5:E153)</f>
         <v>25610</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="29" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="C30" s="47" t="n">
         <f aca="false">C27+C28-C29</f>
@@ -8048,7 +8087,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="29" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="C31" s="48" t="n">
         <v>58805</v>
@@ -8056,7 +8095,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="39" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="C32" s="49" t="n">
         <f aca="false">C30-C31</f>
@@ -8065,7 +8104,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="27" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="C33" s="27"/>
       <c r="D33" s="27"/>
@@ -8106,7 +8145,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8115,7 +8154,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -8124,206 +8163,206 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>29</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="C6" s="14" t="s">
+        <v>454</v>
+      </c>
+      <c r="D6" s="17" t="s">
         <v>450</v>
       </c>
-      <c r="D6" s="17" t="s">
-        <v>446</v>
-      </c>
       <c r="E6" s="14" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="C15" s="14" t="s">
+        <v>485</v>
+      </c>
+      <c r="D15" s="18" t="s">
         <v>481</v>
       </c>
-      <c r="D15" s="18" t="s">
-        <v>477</v>
-      </c>
       <c r="E15" s="14" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: project update 2026-10-02 -- work restarted Sep 24 with new crew, Sep 25 EUR3,000 withdrawal logged (Kairis EUR2,350 paid, balance EUR4,400), Sep 29 batch + electricity meter items Committed
</commit_message>
<xml_diff>
--- a/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
+++ b/Budget/Ag_Nikolaos_Balance_Sheet.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1508" uniqueCount="487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1571" uniqueCount="506">
   <si>
     <t xml:space="preserve">Ag. Nikolaos Home — Project Balance Sheet</t>
   </si>
@@ -791,6 +791,18 @@
     <t xml:space="preserve">Kairis - cash payment toward outstanding materials debt (remainder applied to next SikaGrout order)</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-09-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kairis - cash payment toward SikaGrout order balance (Vicky Sep 29: balance now EUR4,400 after this payment)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remainder of Sep 25 EUR3,000 NBG withdrawal - cash float, allocation TBC (nails/steel strips ~EUR45, mixer petrol; possibly water fee EUR400 / ELEC deposit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vicky (cash float)</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026-06-28</t>
   </si>
   <si>
@@ -863,7 +875,7 @@
     <t xml:space="preserve">2026-07-11</t>
   </si>
   <si>
-    <t xml:space="preserve">Kairis - next SikaGrout order (200 bags) + 20 steel bars - approved by Yael, not yet placed (EUR7,740 minus EUR1,010 applied from Jul23/29 payments)</t>
+    <t xml:space="preserve">Kairis - SikaGrout HP340 order (200 bags) + steel - partly delivered Sep; outstanding balance per Vicky Sep 29 EUR4,400 incl. EUR45 old balance (EUR1,000 payment planned Sep 29, unconfirmed)</t>
   </si>
   <si>
     <t xml:space="preserve">Kairis - partial payment toward column/beam debt</t>
@@ -881,6 +893,39 @@
     <t xml:space="preserve">pending</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-09-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Workers wages - week of Sep 21-27 (crew back on site Sep 24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reinforcement steel, column ties, 15x D16 6m connecting bars + nails</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Petrol for concrete mixer (column pour)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electricity provider - 50% advance to reactivate 1969 meter + relocate to lower entrance (incl. install permit + supply approval); Vicky paid Sep 26, to be covered by Sep 29 withdrawal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electricity provider</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electricity provider - remaining 50% for meter reactivation/relocation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electricity bill (meter still in Anagnostou name) - Vicky to hand cash to Stathis Oct 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anagnostou (Stathis)</t>
+  </si>
+  <si>
     <t xml:space="preserve">PAID — total</t>
   </si>
   <si>
@@ -1488,6 +1533,18 @@
   </si>
   <si>
     <t xml:space="preserve">Ask Vicky to confirm — either an ATM withdrawal that ran ahead of itemized expenses, or a payment not yet reported in the WhatsApp group.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rolling bridge residual -EUR2,212.06 (Oct 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anchor balance (EUR58,805) is from 29-Jul and predates the 25-Sep EUR3,000 withdrawal now logged as Paid (EUR2,350 Kairis + EUR650 unallocated float). Kobi said ~EUR58K on 24-Sep (approx, not used as anchor). Residual moved by exactly the EUR3,000 -- anchor staleness, not missing money.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get a fresh exact NBG spot balance; also confirm whether the 29-Sep EUR3,000 withdrawal happened (its items are still Committed) and how the EUR650 float was spent.</t>
   </si>
 </sst>
 </file>
@@ -2256,8 +2313,8 @@
         <v>10</v>
       </c>
       <c r="B10" s="9" t="n">
-        <f aca="false">'Renovation Ledger'!E154</f>
-        <v>99161.47</v>
+        <f aca="false">'Renovation Ledger'!E162</f>
+        <v>102161.47</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>11</v>
@@ -2268,8 +2325,8 @@
         <v>12</v>
       </c>
       <c r="B11" s="10" t="n">
-        <f aca="false">'Renovation Ledger'!E155</f>
-        <v>20578</v>
+        <f aca="false">'Renovation Ledger'!E163</f>
+        <v>20635</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>13</v>
@@ -2280,8 +2337,8 @@
         <v>14</v>
       </c>
       <c r="B12" s="5" t="n">
-        <f aca="false">'Property Acquisition 2025'!D19+'Renovation Ledger'!E154</f>
-        <v>270870.47</v>
+        <f aca="false">'Property Acquisition 2025'!D19+'Renovation Ledger'!E162</f>
+        <v>273870.47</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>15</v>
@@ -2339,7 +2396,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I157"/>
+  <dimension ref="A1:I165"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="13"/>
@@ -6146,7 +6203,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="14" t="s">
         <v>254</v>
       </c>
@@ -6160,7 +6217,7 @@
         <v>34</v>
       </c>
       <c r="E134" s="15" t="n">
-        <v>1500</v>
+        <v>2350</v>
       </c>
       <c r="F134" s="16" t="s">
         <v>35</v>
@@ -6172,24 +6229,24 @@
         <v>37</v>
       </c>
       <c r="I134" s="14" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="14" t="s">
         <v>254</v>
       </c>
       <c r="B135" s="14" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="C135" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="D135" s="14" t="s">
         <v>257</v>
       </c>
-      <c r="D135" s="14" t="s">
-        <v>111</v>
-      </c>
       <c r="E135" s="15" t="n">
-        <v>200</v>
+        <v>650</v>
       </c>
       <c r="F135" s="16" t="s">
         <v>35</v>
@@ -6201,24 +6258,24 @@
         <v>37</v>
       </c>
       <c r="I135" s="14" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="14" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B136" s="14" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="C136" s="14" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D136" s="14" t="s">
-        <v>259</v>
+        <v>34</v>
       </c>
       <c r="E136" s="15" t="n">
-        <v>250</v>
+        <v>1500</v>
       </c>
       <c r="F136" s="16" t="s">
         <v>35</v>
@@ -6230,53 +6287,53 @@
         <v>37</v>
       </c>
       <c r="I136" s="14" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="14" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B137" s="14" t="s">
-        <v>51</v>
+        <v>106</v>
       </c>
       <c r="C137" s="14" t="s">
+        <v>261</v>
+      </c>
+      <c r="D137" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E137" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="F137" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G137" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H137" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="I137" s="14" t="s">
         <v>260</v>
-      </c>
-      <c r="D137" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="E137" s="15" t="n">
-        <v>50</v>
-      </c>
-      <c r="F137" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="G137" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="H137" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="I137" s="14" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="14" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B138" s="14" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="C138" s="14" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D138" s="14" t="s">
-        <v>222</v>
+        <v>263</v>
       </c>
       <c r="E138" s="15" t="n">
-        <v>40</v>
+        <v>250</v>
       </c>
       <c r="F138" s="16" t="s">
         <v>35</v>
@@ -6288,24 +6345,24 @@
         <v>37</v>
       </c>
       <c r="I138" s="14" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="14" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B139" s="14" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="C139" s="14" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D139" s="14" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E139" s="15" t="n">
-        <v>2600</v>
+        <v>50</v>
       </c>
       <c r="F139" s="16" t="s">
         <v>35</v>
@@ -6317,24 +6374,24 @@
         <v>37</v>
       </c>
       <c r="I139" s="14" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="14" t="s">
-        <v>138</v>
+        <v>258</v>
       </c>
       <c r="B140" s="14" t="s">
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="C140" s="14" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D140" s="14" t="s">
-        <v>81</v>
+        <v>222</v>
       </c>
       <c r="E140" s="15" t="n">
-        <v>9500</v>
+        <v>40</v>
       </c>
       <c r="F140" s="16" t="s">
         <v>35</v>
@@ -6342,37 +6399,41 @@
       <c r="G140" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H140" s="18" t="s">
-        <v>264</v>
-      </c>
-      <c r="I140" s="14"/>
+      <c r="H140" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="I140" s="14" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="14" t="s">
-        <v>138</v>
+        <v>258</v>
       </c>
       <c r="B141" s="14" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C141" s="14" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D141" s="14" t="s">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="E141" s="15" t="n">
-        <v>1000</v>
+        <v>2600</v>
       </c>
       <c r="F141" s="16" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="G141" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H141" s="18" t="s">
-        <v>264</v>
-      </c>
-      <c r="I141" s="14"/>
+      <c r="H141" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="I141" s="14" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="14" t="s">
@@ -6382,22 +6443,22 @@
         <v>43</v>
       </c>
       <c r="C142" s="14" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D142" s="14" t="s">
         <v>81</v>
       </c>
       <c r="E142" s="15" t="n">
-        <v>750</v>
+        <v>9500</v>
       </c>
       <c r="F142" s="16" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="G142" s="16" t="s">
         <v>36</v>
       </c>
       <c r="H142" s="18" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="I142" s="14"/>
     </row>
@@ -6409,7 +6470,7 @@
         <v>43</v>
       </c>
       <c r="C143" s="14" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D143" s="14" t="s">
         <v>81</v>
@@ -6418,13 +6479,13 @@
         <v>1000</v>
       </c>
       <c r="F143" s="16" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="G143" s="16" t="s">
         <v>36</v>
       </c>
       <c r="H143" s="18" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="I143" s="14"/>
     </row>
@@ -6433,43 +6494,43 @@
         <v>138</v>
       </c>
       <c r="B144" s="14" t="s">
-        <v>123</v>
+        <v>43</v>
       </c>
       <c r="C144" s="14" t="s">
+        <v>270</v>
+      </c>
+      <c r="D144" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="E144" s="15" t="n">
+        <v>750</v>
+      </c>
+      <c r="F144" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="G144" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H144" s="18" t="s">
         <v>268</v>
-      </c>
-      <c r="D144" s="14" t="s">
-        <v>269</v>
-      </c>
-      <c r="E144" s="15" t="n">
-        <v>550</v>
-      </c>
-      <c r="F144" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="G144" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="H144" s="18" t="s">
-        <v>264</v>
       </c>
       <c r="I144" s="14"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="14" t="s">
-        <v>203</v>
+        <v>138</v>
       </c>
       <c r="B145" s="14" t="s">
-        <v>82</v>
+        <v>43</v>
       </c>
       <c r="C145" s="14" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D145" s="14" t="s">
-        <v>163</v>
+        <v>81</v>
       </c>
       <c r="E145" s="15" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="F145" s="16" t="s">
         <v>35</v>
@@ -6478,25 +6539,25 @@
         <v>36</v>
       </c>
       <c r="H145" s="18" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="I145" s="14"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="14" t="s">
-        <v>243</v>
+        <v>138</v>
       </c>
       <c r="B146" s="14" t="s">
-        <v>77</v>
+        <v>123</v>
       </c>
       <c r="C146" s="14" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D146" s="14" t="s">
-        <v>88</v>
+        <v>273</v>
       </c>
       <c r="E146" s="15" t="n">
-        <v>1865</v>
+        <v>550</v>
       </c>
       <c r="F146" s="16" t="s">
         <v>35</v>
@@ -6504,28 +6565,26 @@
       <c r="G146" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H146" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="I146" s="14" t="s">
-        <v>243</v>
-      </c>
+      <c r="H146" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="I146" s="14"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="14" t="s">
-        <v>272</v>
+        <v>203</v>
       </c>
       <c r="B147" s="14" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C147" s="14" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D147" s="14" t="s">
-        <v>88</v>
+        <v>163</v>
       </c>
       <c r="E147" s="15" t="n">
-        <v>1990</v>
+        <v>600</v>
       </c>
       <c r="F147" s="16" t="s">
         <v>35</v>
@@ -6533,55 +6592,55 @@
       <c r="G147" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H147" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="I147" s="14" t="s">
-        <v>272</v>
-      </c>
+      <c r="H147" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="I147" s="14"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="14" t="s">
-        <v>226</v>
+        <v>243</v>
       </c>
       <c r="B148" s="14" t="s">
         <v>77</v>
       </c>
       <c r="C148" s="14" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D148" s="14" t="s">
         <v>88</v>
       </c>
       <c r="E148" s="15" t="n">
-        <v>3</v>
+        <v>1865</v>
       </c>
       <c r="F148" s="16" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="G148" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H148" s="18" t="s">
-        <v>264</v>
-      </c>
-      <c r="I148" s="14"/>
+      <c r="H148" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="I148" s="14" t="s">
+        <v>243</v>
+      </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="14" t="s">
-        <v>241</v>
+        <v>276</v>
       </c>
       <c r="B149" s="14" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="C149" s="14" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D149" s="14" t="s">
-        <v>34</v>
+        <v>88</v>
       </c>
       <c r="E149" s="15" t="n">
-        <v>150</v>
+        <v>1990</v>
       </c>
       <c r="F149" s="16" t="s">
         <v>35</v>
@@ -6593,51 +6652,51 @@
         <v>37</v>
       </c>
       <c r="I149" s="14" t="s">
-        <v>243</v>
+        <v>276</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="14" t="s">
-        <v>209</v>
+        <v>226</v>
       </c>
       <c r="B150" s="14" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="C150" s="14" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D150" s="14" t="s">
-        <v>34</v>
+        <v>88</v>
       </c>
       <c r="E150" s="15" t="n">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="F150" s="16" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="G150" s="16" t="s">
         <v>36</v>
       </c>
       <c r="H150" s="18" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="I150" s="14"/>
     </row>
-    <row r="151" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="14" t="s">
-        <v>277</v>
+        <v>241</v>
       </c>
       <c r="B151" s="14" t="s">
         <v>51</v>
       </c>
       <c r="C151" s="14" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D151" s="14" t="s">
         <v>34</v>
       </c>
       <c r="E151" s="15" t="n">
-        <v>6730</v>
+        <v>150</v>
       </c>
       <c r="F151" s="16" t="s">
         <v>35</v>
@@ -6645,26 +6704,28 @@
       <c r="G151" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H151" s="18" t="s">
-        <v>264</v>
-      </c>
-      <c r="I151" s="14"/>
+      <c r="H151" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="I151" s="14" t="s">
+        <v>243</v>
+      </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="14" t="s">
-        <v>272</v>
+        <v>209</v>
       </c>
       <c r="B152" s="14" t="s">
         <v>51</v>
       </c>
       <c r="C152" s="14" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D152" s="14" t="s">
         <v>34</v>
       </c>
       <c r="E152" s="15" t="n">
-        <v>1000</v>
+        <v>45</v>
       </c>
       <c r="F152" s="16" t="s">
         <v>35</v>
@@ -6672,73 +6733,289 @@
       <c r="G152" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H152" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="I152" s="14" t="s">
-        <v>272</v>
-      </c>
+      <c r="H152" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="I152" s="14"/>
     </row>
     <row r="153" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="14" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B153" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C153" s="14" t="s">
+        <v>282</v>
+      </c>
+      <c r="D153" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E153" s="15" t="n">
+        <v>4355</v>
+      </c>
+      <c r="F153" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G153" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H153" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="I153" s="14"/>
+    </row>
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="14" t="s">
+        <v>276</v>
+      </c>
+      <c r="B154" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C154" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="D154" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E154" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F154" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G154" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H154" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="I154" s="14" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="155" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="B155" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="C153" s="14" t="s">
-        <v>281</v>
-      </c>
-      <c r="D153" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="E153" s="15" t="n">
+      <c r="C155" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="D155" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="E155" s="15" t="n">
         <v>400</v>
       </c>
-      <c r="F153" s="16" t="s">
-        <v>283</v>
-      </c>
-      <c r="G153" s="16" t="s">
+      <c r="F155" s="16" t="s">
+        <v>287</v>
+      </c>
+      <c r="G155" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="H153" s="18" t="s">
-        <v>264</v>
-      </c>
-      <c r="I153" s="14"/>
-    </row>
-    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D154" s="19" t="s">
-        <v>284</v>
-      </c>
-      <c r="E154" s="20" t="n">
-        <f aca="false">SUMIF(H5:H153,"Paid",E5:E153)</f>
-        <v>99161.47</v>
-      </c>
-    </row>
-    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D155" s="19" t="s">
-        <v>285</v>
-      </c>
-      <c r="E155" s="21" t="n">
-        <f aca="false">SUMIF(H5:H153,"Committed",E5:E153)</f>
-        <v>20578</v>
-      </c>
-    </row>
-    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D156" s="22" t="s">
-        <v>286</v>
-      </c>
-      <c r="E156" s="23" t="n">
-        <f aca="false">SUMIFS(E5:E153,H5:H153,"Paid",G5:G153,"Yes")</f>
-        <v>97133.92</v>
-      </c>
-    </row>
-    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D157" s="22" t="s">
-        <v>287</v>
-      </c>
-      <c r="E157" s="23" t="n">
-        <f aca="false">SUMIFS(E5:E153,H5:H153,"Paid",G5:G153,"No")</f>
+      <c r="H155" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="I155" s="14"/>
+    </row>
+    <row r="156" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="B156" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C156" s="14" t="s">
+        <v>289</v>
+      </c>
+      <c r="D156" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="E156" s="15" t="n">
+        <v>950</v>
+      </c>
+      <c r="F156" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G156" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H156" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="I156" s="14"/>
+    </row>
+    <row r="157" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="B157" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C157" s="14" t="s">
+        <v>290</v>
+      </c>
+      <c r="D157" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="E157" s="15" t="n">
+        <v>750</v>
+      </c>
+      <c r="F157" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G157" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H157" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="I157" s="14"/>
+    </row>
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="B158" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C158" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="D158" s="14" t="s">
+        <v>245</v>
+      </c>
+      <c r="E158" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="F158" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G158" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H158" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="I158" s="14"/>
+    </row>
+    <row r="159" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="14" t="s">
+        <v>292</v>
+      </c>
+      <c r="B159" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C159" s="14" t="s">
+        <v>293</v>
+      </c>
+      <c r="D159" s="14" t="s">
+        <v>294</v>
+      </c>
+      <c r="E159" s="15" t="n">
+        <v>250</v>
+      </c>
+      <c r="F159" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G159" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H159" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="I159" s="14"/>
+    </row>
+    <row r="160" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="14" t="s">
+        <v>292</v>
+      </c>
+      <c r="B160" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C160" s="14" t="s">
+        <v>295</v>
+      </c>
+      <c r="D160" s="14" t="s">
+        <v>294</v>
+      </c>
+      <c r="E160" s="15" t="n">
+        <v>250</v>
+      </c>
+      <c r="F160" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G160" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H160" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="I160" s="14"/>
+    </row>
+    <row r="161" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="B161" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C161" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="D161" s="14" t="s">
+        <v>298</v>
+      </c>
+      <c r="E161" s="15" t="n">
+        <v>192</v>
+      </c>
+      <c r="F161" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G161" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H161" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="I161" s="14"/>
+    </row>
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D162" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="E162" s="20" t="n">
+        <f aca="false">SUMIF(H5:H161,"Paid",E5:E161)</f>
+        <v>102161.47</v>
+      </c>
+    </row>
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D163" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="E163" s="21" t="n">
+        <f aca="false">SUMIF(H5:H161,"Committed",E5:E161)</f>
+        <v>20635</v>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D164" s="22" t="s">
+        <v>301</v>
+      </c>
+      <c r="E164" s="23" t="n">
+        <f aca="false">SUMIFS(E5:E161,H5:H161,"Paid",G5:G161,"Yes")</f>
+        <v>100133.92</v>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D165" s="22" t="s">
+        <v>302</v>
+      </c>
+      <c r="E165" s="23" t="n">
+        <f aca="false">SUMIFS(E5:E161,H5:H161,"Paid",G5:G161,"No")</f>
         <v>2027.55</v>
       </c>
     </row>
@@ -6774,7 +7051,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>288</v>
+        <v>303</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6783,7 +7060,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>289</v>
+        <v>304</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6792,33 +7069,33 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>290</v>
+        <v>305</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>291</v>
+        <v>306</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>292</v>
+        <v>307</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>293</v>
+        <v>308</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="B5" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>295</v>
+        <v>310</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>296</v>
+        <v>311</v>
       </c>
       <c r="E5" s="17" t="s">
         <v>36</v>
@@ -6826,16 +7103,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="B6" s="24" t="n">
         <v>15000</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>297</v>
+        <v>312</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>298</v>
+        <v>313</v>
       </c>
       <c r="E6" s="17" t="s">
         <v>36</v>
@@ -6843,16 +7120,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>299</v>
+        <v>314</v>
       </c>
       <c r="B7" s="24" t="n">
         <v>130000</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>300</v>
+        <v>315</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>301</v>
+        <v>316</v>
       </c>
       <c r="E7" s="17" t="s">
         <v>36</v>
@@ -6860,16 +7137,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>302</v>
+        <v>317</v>
       </c>
       <c r="B8" s="24" t="n">
         <v>10000</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>303</v>
+        <v>318</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>304</v>
+        <v>319</v>
       </c>
       <c r="E8" s="17" t="s">
         <v>36</v>
@@ -6877,16 +7154,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>305</v>
+        <v>320</v>
       </c>
       <c r="B9" s="24" t="n">
         <v>20000</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>306</v>
+        <v>321</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>307</v>
+        <v>322</v>
       </c>
       <c r="E9" s="17" t="s">
         <v>36</v>
@@ -6894,16 +7171,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>308</v>
+        <v>323</v>
       </c>
       <c r="B10" s="24" t="n">
         <v>70000</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>309</v>
+        <v>324</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>310</v>
+        <v>325</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>36</v>
@@ -6911,16 +7188,16 @@
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>311</v>
+        <v>326</v>
       </c>
       <c r="B11" s="24" t="n">
         <v>2000</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>313</v>
+        <v>328</v>
       </c>
       <c r="E11" s="18" t="s">
         <v>183</v>
@@ -6928,16 +7205,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>314</v>
+        <v>329</v>
       </c>
       <c r="B12" s="24" t="n">
         <v>50000</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>316</v>
+        <v>331</v>
       </c>
       <c r="E12" s="17" t="s">
         <v>36</v>
@@ -6945,7 +7222,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="25" t="s">
-        <v>317</v>
+        <v>332</v>
       </c>
       <c r="B13" s="26" t="n">
         <f aca="false">SUMIF(E5:E12,"Yes",B5:B12)</f>
@@ -6954,7 +7231,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="27" t="s">
-        <v>318</v>
+        <v>333</v>
       </c>
       <c r="B15" s="27"/>
       <c r="C15" s="27"/>
@@ -6963,7 +7240,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="27" t="s">
-        <v>319</v>
+        <v>334</v>
       </c>
       <c r="B16" s="27"/>
       <c r="C16" s="27"/>
@@ -7005,7 +7282,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>320</v>
+        <v>335</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7014,7 +7291,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>321</v>
+        <v>336</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7023,13 +7300,13 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>323</v>
+        <v>338</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>324</v>
+        <v>339</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>26</v>
@@ -7038,18 +7315,18 @@
         <v>28</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>325</v>
+        <v>340</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>326</v>
+        <v>341</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>327</v>
+        <v>342</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="D5" s="24" t="n">
         <v>18500</v>
@@ -7058,18 +7335,18 @@
         <v>36</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>329</v>
+        <v>344</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>330</v>
+        <v>345</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>331</v>
+        <v>346</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>332</v>
+        <v>347</v>
       </c>
       <c r="D6" s="24" t="n">
         <v>107000</v>
@@ -7078,18 +7355,18 @@
         <v>36</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>333</v>
+        <v>348</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>330</v>
+        <v>345</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>334</v>
+        <v>349</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="D7" s="24" t="n">
         <v>19731</v>
@@ -7098,18 +7375,18 @@
         <v>36</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>335</v>
+        <v>350</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>336</v>
+        <v>351</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>337</v>
+        <v>352</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>338</v>
+        <v>353</v>
       </c>
       <c r="D8" s="24" t="n">
         <v>7410</v>
@@ -7118,18 +7395,18 @@
         <v>36</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>339</v>
+        <v>354</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>340</v>
+        <v>355</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>341</v>
+        <v>356</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>342</v>
+        <v>357</v>
       </c>
       <c r="D9" s="24" t="n">
         <v>4350</v>
@@ -7138,15 +7415,15 @@
         <v>36</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>343</v>
+        <v>358</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>340</v>
+        <v>355</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>344</v>
+        <v>359</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>150</v>
@@ -7158,15 +7435,15 @@
         <v>36</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>345</v>
+        <v>360</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>340</v>
+        <v>355</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>346</v>
+        <v>361</v>
       </c>
       <c r="C11" s="14" t="s">
         <v>150</v>
@@ -7178,18 +7455,18 @@
         <v>36</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>347</v>
+        <v>362</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>348</v>
+        <v>363</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>349</v>
+        <v>364</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>350</v>
+        <v>365</v>
       </c>
       <c r="D12" s="24" t="n">
         <v>2490</v>
@@ -7198,18 +7475,18 @@
         <v>36</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>335</v>
+        <v>350</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>326</v>
+        <v>341</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>351</v>
+        <v>366</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="D13" s="24" t="n">
         <v>800</v>
@@ -7218,18 +7495,18 @@
         <v>36</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>353</v>
+        <v>368</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>354</v>
+        <v>369</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>355</v>
+        <v>370</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="D14" s="24" t="n">
         <v>520</v>
@@ -7241,13 +7518,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>354</v>
+        <v>369</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>356</v>
+        <v>371</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>357</v>
+        <v>372</v>
       </c>
       <c r="D15" s="24" t="n">
         <v>680</v>
@@ -7259,13 +7536,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>359</v>
+        <v>374</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="D16" s="24" t="n">
         <v>3000</v>
@@ -7274,15 +7551,15 @@
         <v>36</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>361</v>
+        <v>376</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>362</v>
+        <v>377</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>48</v>
@@ -7294,15 +7571,15 @@
         <v>183</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>363</v>
+        <v>378</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>364</v>
+        <v>379</v>
       </c>
       <c r="C18" s="14" t="s">
         <v>48</v>
@@ -7314,12 +7591,12 @@
         <v>183</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>365</v>
+        <v>380</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C19" s="25" t="s">
-        <v>366</v>
+        <v>381</v>
       </c>
       <c r="D19" s="26" t="n">
         <f aca="false">SUM(D5:D18)</f>
@@ -7328,7 +7605,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C20" s="19" t="s">
-        <v>367</v>
+        <v>382</v>
       </c>
       <c r="D20" s="28" t="n">
         <f aca="false">SUMIF(E5:E18,"Yes",D5:D18)</f>
@@ -7337,7 +7614,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="27" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="27"/>
@@ -7378,7 +7655,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>369</v>
+        <v>384</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7387,7 +7664,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7396,10 +7673,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>323</v>
+        <v>338</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>27</v>
@@ -7408,7 +7685,7 @@
         <v>26</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>325</v>
+        <v>340</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7416,7 +7693,7 @@
         <v>170</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>371</v>
+        <v>386</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>182</v>
@@ -7425,7 +7702,7 @@
         <v>614</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>372</v>
+        <v>387</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7433,7 +7710,7 @@
         <v>205</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>373</v>
+        <v>388</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>208</v>
@@ -7442,7 +7719,7 @@
         <v>972.55</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>374</v>
+        <v>389</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7450,7 +7727,7 @@
         <v>212</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>375</v>
+        <v>390</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>182</v>
@@ -7459,7 +7736,7 @@
         <v>286</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>376</v>
+        <v>391</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7467,7 +7744,7 @@
         <v>216</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>377</v>
+        <v>392</v>
       </c>
       <c r="C8" s="14" t="s">
         <v>208</v>
@@ -7476,12 +7753,12 @@
         <v>155</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>378</v>
+        <v>393</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="19" t="s">
-        <v>379</v>
+        <v>394</v>
       </c>
       <c r="D9" s="20" t="n">
         <f aca="false">SUM(D5:D8)</f>
@@ -7490,7 +7767,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>380</v>
+        <v>395</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
@@ -7499,10 +7776,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>323</v>
+        <v>338</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>27</v>
@@ -7511,7 +7788,7 @@
         <v>26</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>325</v>
+        <v>340</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7519,16 +7796,16 @@
         <v>216</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>381</v>
+        <v>396</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>382</v>
+        <v>397</v>
       </c>
       <c r="D13" s="15" t="n">
         <v>972.55</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>383</v>
+        <v>398</v>
       </c>
     </row>
   </sheetData>
@@ -7562,7 +7839,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>384</v>
+        <v>399</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7570,7 +7847,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7581,13 +7858,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>386</v>
+        <v>401</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>387</v>
+        <v>402</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>388</v>
+        <v>403</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7595,14 +7872,14 @@
         <v>38</v>
       </c>
       <c r="B5" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A5,'Renovation Ledger'!H5:H153,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A5,'Renovation Ledger'!H5:H161,"Paid")</f>
         <v>30190</v>
       </c>
       <c r="C5" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>389</v>
+        <v>404</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7610,14 +7887,14 @@
         <v>51</v>
       </c>
       <c r="B6" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A6,'Renovation Ledger'!H5:H153,"Paid")</f>
-        <v>37057.87</v>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A6,'Renovation Ledger'!H5:H161,"Paid")</f>
+        <v>39407.87</v>
       </c>
       <c r="C6" s="24" t="n">
         <v>25000</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>390</v>
+        <v>405</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7625,14 +7902,14 @@
         <v>106</v>
       </c>
       <c r="B7" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A7,'Renovation Ledger'!H5:H153,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A7,'Renovation Ledger'!H5:H161,"Paid")</f>
         <v>7119</v>
       </c>
       <c r="C7" s="24" t="n">
         <v>9000</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>391</v>
+        <v>406</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7640,14 +7917,14 @@
         <v>43</v>
       </c>
       <c r="B8" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A8,'Renovation Ledger'!H5:H153,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A8,'Renovation Ledger'!H5:H161,"Paid")</f>
         <v>2325</v>
       </c>
       <c r="C8" s="24" t="n">
         <v>11250</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>392</v>
+        <v>407</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7655,14 +7932,14 @@
         <v>82</v>
       </c>
       <c r="B9" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A9,'Renovation Ledger'!H5:H153,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A9,'Renovation Ledger'!H5:H161,"Paid")</f>
         <v>4300</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>6000</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>393</v>
+        <v>408</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7670,14 +7947,14 @@
         <v>104</v>
       </c>
       <c r="B10" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A10,'Renovation Ledger'!H5:H153,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A10,'Renovation Ledger'!H5:H161,"Paid")</f>
         <v>4225</v>
       </c>
       <c r="C10" s="24" t="n">
         <v>4500</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>394</v>
+        <v>409</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7685,14 +7962,14 @@
         <v>123</v>
       </c>
       <c r="B11" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A11,'Renovation Ledger'!H5:H153,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A11,'Renovation Ledger'!H5:H161,"Paid")</f>
         <v>1550</v>
       </c>
       <c r="C11" s="24" t="n">
         <v>18700</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>395</v>
+        <v>410</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7700,14 +7977,14 @@
         <v>32</v>
       </c>
       <c r="B12" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A12,'Renovation Ledger'!H5:H153,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A12,'Renovation Ledger'!H5:H161,"Paid")</f>
         <v>2097</v>
       </c>
       <c r="C12" s="24" t="n">
         <v>2000</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>396</v>
+        <v>411</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7715,14 +7992,14 @@
         <v>213</v>
       </c>
       <c r="B13" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A13,'Renovation Ledger'!H5:H153,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A13,'Renovation Ledger'!H5:H161,"Paid")</f>
         <v>286</v>
       </c>
       <c r="C13" s="24" t="n">
         <v>25500</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7730,14 +8007,14 @@
         <v>219</v>
       </c>
       <c r="B14" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A14,'Renovation Ledger'!H5:H153,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A14,'Renovation Ledger'!H5:H161,"Paid")</f>
         <v>905</v>
       </c>
       <c r="C14" s="24" t="n">
         <v>1000</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7745,14 +8022,14 @@
         <v>77</v>
       </c>
       <c r="B15" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A15,'Renovation Ledger'!H5:H153,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A15,'Renovation Ledger'!H5:H161,"Paid")</f>
         <v>7666</v>
       </c>
       <c r="C15" s="24" t="n">
         <v>11350</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7760,14 +8037,14 @@
         <v>95</v>
       </c>
       <c r="B16" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A16,'Renovation Ledger'!H5:H153,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A16,'Renovation Ledger'!H5:H161,"Paid")</f>
         <v>300</v>
       </c>
       <c r="C16" s="24" t="n">
         <v>5000</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7775,7 +8052,7 @@
         <v>71</v>
       </c>
       <c r="B17" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A17,'Renovation Ledger'!H5:H153,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A17,'Renovation Ledger'!H5:H161,"Paid")</f>
         <v>270</v>
       </c>
       <c r="C17" s="24" t="n">
@@ -7790,14 +8067,14 @@
         <v>46</v>
       </c>
       <c r="B18" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A18,'Renovation Ledger'!H5:H153,"Paid")</f>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A18,'Renovation Ledger'!H5:H161,"Paid")</f>
         <v>770.6</v>
       </c>
       <c r="C18" s="24" t="n">
         <v>500</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>401</v>
+        <v>416</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7805,23 +8082,23 @@
         <v>66</v>
       </c>
       <c r="B19" s="15" t="n">
-        <f aca="false">SUMIFS('Renovation Ledger'!E5:E153,'Renovation Ledger'!B5:B153,A19,'Renovation Ledger'!H5:H153,"Paid")</f>
-        <v>100</v>
+        <f aca="false">SUMIFS('Renovation Ledger'!E5:E161,'Renovation Ledger'!B5:B161,A19,'Renovation Ledger'!H5:H161,"Paid")</f>
+        <v>750</v>
       </c>
       <c r="C19" s="24" t="n">
         <v>300</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>402</v>
+        <v>417</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="29" t="s">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="B20" s="20" t="n">
         <f aca="false">SUM(B5:B19)</f>
-        <v>99161.47</v>
+        <v>102161.47</v>
       </c>
       <c r="C20" s="28" t="n">
         <f aca="false">SUM(C5:C19)</f>
@@ -7859,7 +8136,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>404</v>
+        <v>419</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7867,7 +8144,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>405</v>
+        <v>420</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7875,106 +8152,106 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="30" t="s">
-        <v>406</v>
+        <v>421</v>
       </c>
       <c r="C5" s="31" t="n">
         <v>21066.81</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>407</v>
+        <v>422</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="33" t="s">
-        <v>408</v>
+        <v>423</v>
       </c>
       <c r="C6" s="34" t="n">
         <v>230000</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>409</v>
+        <v>424</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="35" t="s">
-        <v>410</v>
+        <v>425</v>
       </c>
       <c r="C7" s="36" t="n">
         <v>-139459.28</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>411</v>
+        <v>426</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="35" t="s">
-        <v>412</v>
+        <v>427</v>
       </c>
       <c r="C8" s="36" t="n">
         <v>-6350</v>
       </c>
       <c r="D8" s="32" t="s">
-        <v>413</v>
+        <v>428</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="35" t="s">
-        <v>414</v>
+        <v>429</v>
       </c>
       <c r="C9" s="36" t="n">
         <v>-64730</v>
       </c>
       <c r="D9" s="32" t="s">
-        <v>415</v>
+        <v>430</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="35" t="s">
-        <v>416</v>
+        <v>431</v>
       </c>
       <c r="C10" s="36" t="n">
         <v>-4494.92</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>417</v>
+        <v>432</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="35" t="s">
-        <v>418</v>
+        <v>433</v>
       </c>
       <c r="C11" s="36" t="n">
         <v>-711</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>419</v>
+        <v>434</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="35" t="s">
-        <v>420</v>
+        <v>435</v>
       </c>
       <c r="C12" s="36" t="n">
         <v>-104.17</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>421</v>
+        <v>436</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="35" t="s">
-        <v>422</v>
+        <v>437</v>
       </c>
       <c r="C13" s="36" t="n">
         <v>-14.5</v>
       </c>
       <c r="D13" s="32" t="s">
-        <v>423</v>
+        <v>438</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="29" t="s">
-        <v>424</v>
+        <v>439</v>
       </c>
       <c r="C14" s="37" t="n">
         <f aca="false">SUM(C5:C13)</f>
@@ -7983,7 +8260,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="29" t="s">
-        <v>425</v>
+        <v>440</v>
       </c>
       <c r="C15" s="38" t="n">
         <v>35202.94</v>
@@ -7991,7 +8268,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="39" t="s">
-        <v>426</v>
+        <v>441</v>
       </c>
       <c r="C16" s="40" t="n">
         <f aca="false">C14-C15</f>
@@ -8000,21 +8277,21 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="29" t="s">
-        <v>427</v>
+        <v>442</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="41" t="s">
-        <v>428</v>
+        <v>443</v>
       </c>
       <c r="C19" s="42" t="n">
-        <f aca="false">'Renovation Ledger'!E156</f>
-        <v>97133.92</v>
+        <f aca="false">'Renovation Ledger'!E164</f>
+        <v>100133.92</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="41" t="s">
-        <v>429</v>
+        <v>444</v>
       </c>
       <c r="C20" s="42" t="n">
         <v>69935.92</v>
@@ -8022,37 +8299,37 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="43" t="s">
-        <v>430</v>
+        <v>445</v>
       </c>
       <c r="C21" s="44" t="n">
-        <f aca="false">'Renovation Ledger'!E156-69935.92</f>
-        <v>27198</v>
+        <f aca="false">'Renovation Ledger'!E164-69935.92</f>
+        <v>30198</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="45" t="s">
-        <v>431</v>
+        <v>446</v>
       </c>
       <c r="C23" s="45"/>
       <c r="D23" s="45"/>
     </row>
     <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="45" t="s">
-        <v>432</v>
+        <v>447</v>
       </c>
       <c r="C24" s="45"/>
       <c r="D24" s="45"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="46" t="s">
-        <v>433</v>
+        <v>448</v>
       </c>
       <c r="C26" s="46"/>
       <c r="D26" s="46"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="41" t="s">
-        <v>434</v>
+        <v>449</v>
       </c>
       <c r="C27" s="42" t="n">
         <v>35202.94</v>
@@ -8060,7 +8337,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="41" t="s">
-        <v>435</v>
+        <v>450</v>
       </c>
       <c r="C28" s="42" t="n">
         <f aca="false">SUMPRODUCT(('Funding (NBG Deposits)'!A5:A12&gt;"2026-06-25")*('Funding (NBG Deposits)'!E5:E12="Yes")*'Funding (NBG Deposits)'!B5:B12)</f>
@@ -8069,25 +8346,25 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="41" t="s">
-        <v>436</v>
+        <v>451</v>
       </c>
       <c r="C29" s="42" t="n">
-        <f aca="false">SUMPRODUCT(('Renovation Ledger'!I5:I153&gt;"2026-06-25")*('Renovation Ledger'!H5:H153="Paid")*('Renovation Ledger'!G5:G153="Yes")*'Renovation Ledger'!E5:E153)</f>
-        <v>25610</v>
+        <f aca="false">SUMPRODUCT(('Renovation Ledger'!I5:I161&gt;"2026-06-25")*('Renovation Ledger'!H5:H161="Paid")*('Renovation Ledger'!G5:G161="Yes")*'Renovation Ledger'!E5:E161)</f>
+        <v>28610</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="29" t="s">
-        <v>437</v>
+        <v>452</v>
       </c>
       <c r="C30" s="47" t="n">
         <f aca="false">C27+C28-C29</f>
-        <v>59592.94</v>
+        <v>56592.94</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="29" t="s">
-        <v>438</v>
+        <v>453</v>
       </c>
       <c r="C31" s="48" t="n">
         <v>58805</v>
@@ -8095,16 +8372,16 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="39" t="s">
-        <v>439</v>
+        <v>454</v>
       </c>
       <c r="C32" s="49" t="n">
         <f aca="false">C30-C31</f>
-        <v>787.940000000002</v>
+        <v>-2212.06</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="27" t="s">
-        <v>440</v>
+        <v>455</v>
       </c>
       <c r="C33" s="27"/>
       <c r="D33" s="27"/>
@@ -8133,7 +8410,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -8145,7 +8422,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>441</v>
+        <v>456</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8154,7 +8431,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>442</v>
+        <v>457</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -8163,206 +8440,223 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>443</v>
+        <v>458</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>444</v>
+        <v>459</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>445</v>
+        <v>460</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>29</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>446</v>
+        <v>461</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>447</v>
+        <v>462</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>448</v>
+        <v>463</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>449</v>
+        <v>464</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>450</v>
+        <v>465</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>451</v>
+        <v>466</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>452</v>
+        <v>467</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>453</v>
+        <v>468</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>454</v>
+        <v>469</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>450</v>
+        <v>465</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>455</v>
+        <v>470</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>456</v>
+        <v>471</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>457</v>
+        <v>472</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>458</v>
+        <v>473</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>450</v>
+        <v>465</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>459</v>
+        <v>474</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>460</v>
+        <v>475</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>461</v>
+        <v>476</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>462</v>
+        <v>477</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>450</v>
+        <v>465</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>451</v>
+        <v>466</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>463</v>
+        <v>478</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>464</v>
+        <v>479</v>
       </c>
       <c r="C9" s="14" t="s">
+        <v>480</v>
+      </c>
+      <c r="D9" s="17" t="s">
         <v>465</v>
       </c>
-      <c r="D9" s="17" t="s">
-        <v>450</v>
-      </c>
       <c r="E9" s="14" t="s">
-        <v>451</v>
+        <v>466</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
+        <v>481</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>482</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>483</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>465</v>
+      </c>
+      <c r="E10" s="14" t="s">
         <v>466</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>467</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>468</v>
-      </c>
-      <c r="D10" s="17" t="s">
-        <v>450</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>451</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>469</v>
+        <v>484</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>470</v>
+        <v>485</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>471</v>
+        <v>486</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>450</v>
+        <v>465</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>451</v>
+        <v>466</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>472</v>
+        <v>487</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>473</v>
+        <v>488</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>474</v>
+        <v>489</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>450</v>
+        <v>465</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>451</v>
+        <v>466</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>475</v>
+        <v>490</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>476</v>
+        <v>491</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>477</v>
+        <v>492</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>450</v>
+        <v>465</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>451</v>
+        <v>466</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>478</v>
+        <v>493</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>479</v>
+        <v>494</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>480</v>
+        <v>495</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>481</v>
+        <v>496</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>482</v>
+        <v>497</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>483</v>
+        <v>498</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>484</v>
+        <v>499</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>485</v>
+        <v>500</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>481</v>
+        <v>496</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>486</v>
+        <v>501</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="s">
+        <v>502</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>503</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>504</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>496</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>505</v>
       </c>
     </row>
   </sheetData>

</xml_diff>